<commit_message>
Rediseña el informe de la Práctica 2: paleta azul y carmín, gráficas de estilo artículo y fotografías
- Vientres contiguos en azul y rojo (oposición de fase) en portada y figuras.
- Gráficas con ejes en caja, marcas interiores y leyendas enmarcadas.
- Fotografías del montaje, del estroboscopio y de los modos n = 2 y n = 5.
- Cada sección en una página propia.
- Medida n = 5 de la cuerda doble en L1 (0,013 N) anotada como descartada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TJnn6BdNLSdEVTuuzq6wN7
</commit_message>
<xml_diff>
--- a/practica-2-ondas/ajustes/Ondas_estacionarias.xlsx
+++ b/practica-2-ondas/ajustes/Ondas_estacionarias.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="23">
   <si>
     <t>Cuerda simple en la posición L2</t>
   </si>
@@ -32,6 +32,9 @@
   </si>
   <si>
     <t>T (N)</t>
+  </si>
+  <si>
+    <t>Lambda 2</t>
   </si>
   <si>
     <t>37,6 cm</t>
@@ -135,8 +138,1109 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+  <c:chart>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln cmpd="sng">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:name>Línea de tendencia de serie 1</c:name>
+            <c:spPr>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Hoja 1'!$H$3:$H$7</c:f>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Hoja 1'!$I$3:$I$7</c:f>
+              <c:numCache/>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1552910098"/>
+        <c:axId val="624253450"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1552910098"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC">
+                  <a:alpha val="0"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="624253450"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="624253450"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC">
+                  <a:alpha val="0"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1552910098"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr b="0">
+              <a:solidFill>
+                <a:srgbClr val="1A1A1A"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+  <c:chart>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln cmpd="sng">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:name>Línea de tendencia de serie 1</c:name>
+            <c:spPr>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Hoja 1'!$H$12:$H$17</c:f>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Hoja 1'!$I$12:$I$16</c:f>
+              <c:numCache/>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="676912946"/>
+        <c:axId val="932986082"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="676912946"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC">
+                  <a:alpha val="0"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="932986082"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="932986082"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC">
+                  <a:alpha val="0"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="676912946"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr b="0">
+              <a:solidFill>
+                <a:srgbClr val="1A1A1A"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+  <c:chart>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln cmpd="sng">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:name>Línea de tendencia de serie 1</c:name>
+            <c:spPr>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Hoja 1'!$O$3:$O$7</c:f>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Hoja 1'!$P$3:$P$7</c:f>
+              <c:numCache/>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1488549568"/>
+        <c:axId val="52288460"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1488549568"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC">
+                  <a:alpha val="0"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="52288460"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="52288460"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC">
+                  <a:alpha val="0"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1488549568"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr b="0">
+              <a:solidFill>
+                <a:srgbClr val="1A1A1A"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+  <c:chart>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln cmpd="sng">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:name>Línea de tendencia de serie 1</c:name>
+            <c:spPr>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Hoja 1'!$O$12:$O$16</c:f>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Hoja 1'!$P$12:$P$16</c:f>
+              <c:numCache/>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1084744005"/>
+        <c:axId val="132678525"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1084744005"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC">
+                  <a:alpha val="0"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="132678525"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="132678525"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC">
+                  <a:alpha val="0"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:rPr>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1084744005"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr b="0">
+              <a:solidFill>
+                <a:srgbClr val="1A1A1A"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>609600</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5200650" cy="3257550"/>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart 1" title="Gráfico"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5534025" cy="3457575"/>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 2" title="Gráfico"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>742950</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5600700" cy="3457575"/>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 3" title="Gráfico"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>390525</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5353050" cy="3305175"/>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 4" title="Gráfico"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -352,11 +1456,11 @@
       </c>
       <c r="F1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="2"/>
       <c r="M1" s="2"/>
+      <c r="O1" s="2"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
@@ -374,23 +1478,29 @@
       <c r="H2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="I2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="L2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>6</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F3" s="2">
         <v>43.0</v>
@@ -398,29 +1508,37 @@
       <c r="H3" s="2">
         <v>0.15</v>
       </c>
-      <c r="J3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="K3" s="2">
+      <c r="I3" s="3">
+        <f> (1/43)^2 *(H3/S3)</f>
+        <v>0.6625202812</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M3" s="2">
         <v>43.0</v>
       </c>
-      <c r="M3" s="2">
+      <c r="O3" s="2">
         <v>0.25</v>
       </c>
-      <c r="O3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="P3" s="2" t="s">
+      <c r="P3" s="3">
+        <f> (1/43)^2 *(O3/S3)</f>
+        <v>1.104200469</v>
+      </c>
+      <c r="Q3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="Q3" s="3">
+      <c r="R3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="S3" s="3">
         <f> 0.06*10^(-3)/(49*10^(-2))</f>
         <v>0.0001224489796</v>
       </c>
     </row>
     <row r="4">
       <c r="E4" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F4" s="2">
         <v>43.0</v>
@@ -428,22 +1546,30 @@
       <c r="H4" s="2">
         <v>0.04</v>
       </c>
-      <c r="J4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="K4" s="2">
+      <c r="I4" s="3">
+        <f> (1/43)^2 *(H4/S3)</f>
+        <v>0.176672075</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M4" s="2">
         <v>43.0</v>
       </c>
-      <c r="M4" s="2">
+      <c r="O4" s="2">
         <v>0.07</v>
       </c>
-      <c r="O4" s="2" t="s">
-        <v>12</v>
+      <c r="P4" s="3">
+        <f> (1/43)^2 *(O4/S3)</f>
+        <v>0.3091761312</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="E5" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F5" s="2">
         <v>43.0</v>
@@ -451,25 +1577,33 @@
       <c r="H5" s="2">
         <v>0.02</v>
       </c>
-      <c r="J5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="K5" s="2">
+      <c r="I5" s="3">
+        <f> (1/43)^2 *(H5/S3)</f>
+        <v>0.0883360375</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M5" s="2">
         <v>43.0</v>
       </c>
-      <c r="M5" s="2">
+      <c r="O5" s="2">
         <v>0.03</v>
+      </c>
+      <c r="P5" s="3">
+        <f> (1/43)^2 *(O5/S3)</f>
+        <v>0.1325040562</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F6" s="2">
         <v>43.0</v>
@@ -477,22 +1611,30 @@
       <c r="H6" s="2">
         <v>0.01</v>
       </c>
-      <c r="J6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="K6" s="2">
+      <c r="I6" s="3">
+        <f> (1/43)^2 *(H6/S3)</f>
+        <v>0.04416801875</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" s="2">
         <v>43.0</v>
       </c>
-      <c r="M6" s="2">
+      <c r="O6" s="2">
         <v>0.008</v>
+      </c>
+      <c r="P6" s="3">
+        <f> (1/43)^2 *(O6/S3)</f>
+        <v>0.035334415</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F7" s="2">
         <v>44.0</v>
@@ -500,25 +1642,39 @@
       <c r="H7" s="2">
         <v>0.006</v>
       </c>
-      <c r="J7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="K7" s="2">
+      <c r="I7" s="3">
+        <f> (1/43)^2 *(H7/S3)</f>
+        <v>0.02650081125</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M7" s="2">
         <v>44.0</v>
       </c>
-      <c r="M7" s="2">
+      <c r="O7" s="2">
         <v>0.002</v>
+      </c>
+      <c r="P7" s="3">
+        <f> (1/43)^2 *(O7/S3)</f>
+        <v>0.00883360375</v>
       </c>
     </row>
     <row r="10">
       <c r="E10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J10" s="2" t="s">
         <v>20</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="11">
+      <c r="A11" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="B11" s="3">
+        <v>0.6625202812330989</v>
+      </c>
       <c r="E11" s="2" t="s">
         <v>4</v>
       </c>
@@ -528,19 +1684,28 @@
       <c r="H11" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="I11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="L11" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="M11" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="M11" s="2" t="s">
+      <c r="O11" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="12">
+      <c r="A12" s="2">
+        <v>0.04</v>
+      </c>
+      <c r="B12" s="3">
+        <v>0.17667207499549303</v>
+      </c>
       <c r="E12" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F12" s="2">
         <v>43.0</v>
@@ -548,19 +1713,33 @@
       <c r="H12" s="2">
         <v>0.29</v>
       </c>
-      <c r="J12" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="K12" s="2">
+      <c r="I12" s="3">
+        <f> (1/43)^2 *(H12/(2*S3))</f>
+        <v>0.6404362719</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M12" s="2">
         <v>43.0</v>
       </c>
-      <c r="M12" s="2">
+      <c r="O12" s="2">
         <v>0.5</v>
+      </c>
+      <c r="P12" s="3">
+        <f> (1/43)^2 *(O12/(2*S3))</f>
+        <v>1.104200469</v>
       </c>
     </row>
     <row r="13">
+      <c r="A13" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="B13" s="3">
+        <v>0.08833603749774652</v>
+      </c>
       <c r="E13" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F13" s="2">
         <v>43.0</v>
@@ -568,19 +1747,33 @@
       <c r="H13" s="2">
         <v>0.08</v>
       </c>
-      <c r="J13" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="K13" s="2">
+      <c r="I13" s="3">
+        <f> (1/43)^2 *(H13/(2*S3))</f>
+        <v>0.176672075</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M13" s="2">
         <v>43.0</v>
       </c>
-      <c r="M13" s="2">
+      <c r="O13" s="2">
         <v>0.14</v>
+      </c>
+      <c r="P13" s="3">
+        <f> (1/43)^2 *(O13/(2*S3))</f>
+        <v>0.3091761312</v>
       </c>
     </row>
     <row r="14">
+      <c r="A14" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="B14" s="3">
+        <v>0.04416801874887326</v>
+      </c>
       <c r="E14" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F14" s="2">
         <v>43.0</v>
@@ -588,19 +1781,33 @@
       <c r="H14" s="2">
         <v>0.04</v>
       </c>
-      <c r="J14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="K14" s="2">
+      <c r="I14" s="3">
+        <f> (1/43)^2 *(H14/(2*S3))</f>
+        <v>0.0883360375</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M14" s="2">
         <v>43.0</v>
       </c>
-      <c r="M14" s="2">
+      <c r="O14" s="2">
         <v>0.06</v>
+      </c>
+      <c r="P14" s="3">
+        <f> (1/43)^2 *(O14/(2*S3))</f>
+        <v>0.1325040562</v>
       </c>
     </row>
     <row r="15">
+      <c r="A15" s="2">
+        <v>0.006</v>
+      </c>
+      <c r="B15" s="3">
+        <v>0.026500811249323956</v>
+      </c>
       <c r="E15" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F15" s="2">
         <v>43.0</v>
@@ -608,19 +1815,27 @@
       <c r="H15" s="2">
         <v>0.02</v>
       </c>
-      <c r="J15" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="K15" s="2">
+      <c r="I15" s="3">
+        <f> (1/43)^2 *(H15/(2*S3))</f>
+        <v>0.04416801875</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M15" s="2">
         <v>43.0</v>
       </c>
-      <c r="M15" s="2">
-        <v>0.034</v>
+      <c r="O15" s="2">
+        <v>0.017</v>
+      </c>
+      <c r="P15" s="3">
+        <f> (1/43)^2 *(O15/(2*S3))</f>
+        <v>0.03754281594</v>
       </c>
     </row>
     <row r="16">
       <c r="E16" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F16" s="2">
         <v>43.0</v>
@@ -628,19 +1843,27 @@
       <c r="H16" s="2">
         <v>0.014</v>
       </c>
-      <c r="J16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="K16" s="2">
+      <c r="I16" s="3">
+        <f> (1/43)^2 *(H16/(2*S3))</f>
+        <v>0.03091761312</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M16" s="2">
         <v>43.0</v>
       </c>
-      <c r="M16" s="2">
-        <v>0.036</v>
+      <c r="O16" s="2">
+        <v>0.013</v>
+      </c>
+      <c r="P16" s="3">
+        <f> (1/43)^2 *(O16/(2*S3))</f>
+        <v>0.02870921219</v>
       </c>
     </row>
     <row r="17">
       <c r="E17" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F17" s="2">
         <v>44.0</v>
@@ -648,11 +1871,9 @@
       <c r="H17" s="2">
         <v>0.01</v>
       </c>
-      <c r="J17" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K17" s="2">
-        <v>44.0</v>
+      <c r="I17" s="3">
+        <f> (1/43)^2 *(H17/(2*S3))</f>
+        <v>0.02208400937</v>
       </c>
     </row>
   </sheetData>

</xml_diff>